<commit_message>
Update demo.xlsx with OSCAL-compliant control IDs
- Fixed control ID format to use lowercase and periods instead of parentheses
- Changed AC-17 (02) to ac-17.2 format
- Removed uppercase letters and special characters from control IDs
- File now passes xlsx-to-oscal-cd validation successfully

Signed-off-by: Besjana-Kukaj <beskukaj2004@gmail.com>
</commit_message>
<xml_diff>
--- a/trestle_task_spread_sheet_to_component_definition/demo.xlsx
+++ b/trestle_task_spread_sheet_to_component_definition/demo.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="example_best_practices_controls" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="example_best_practices_controls" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -63,7 +63,7 @@
     <t xml:space="preserve">Check whether the EU supported setting is enabled in account settings</t>
   </si>
   <si>
-    <t xml:space="preserve">CM-2</t>
+    <t xml:space="preserve">CM-02</t>
   </si>
   <si>
     <t xml:space="preserve">SYSTEM</t>
@@ -72,16 +72,16 @@
     <t xml:space="preserve">Check whether Cloudant has no more than # users with the IAM administrator role</t>
   </si>
   <si>
-    <t xml:space="preserve">AC-2: (j)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AC-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AC-5: (b)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AC-6</t>
+    <t xml:space="preserve">AC-02: (j)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC-05: (b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC-06</t>
   </si>
   <si>
     <t xml:space="preserve">CLOUDANT</t>
@@ -189,13 +189,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">AC-17 (2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SC-8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SC-8 (1)</t>
+    <t xml:space="preserve">AC-17 (02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC-08 (01)</t>
   </si>
   <si>
     <t xml:space="preserve">SC-13</t>
@@ -260,13 +260,13 @@
     <t xml:space="preserve">Check whether Virtual Private Cloud (VPC) security groups have no inbound ports open to the internet (0.0.0.0/0)</t>
   </si>
   <si>
-    <t xml:space="preserve">AC-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SC-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SC-7 (3)</t>
+    <t xml:space="preserve">AC-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC-07 (03)</t>
   </si>
   <si>
     <t xml:space="preserve">--</t>
@@ -287,16 +287,16 @@
     <t xml:space="preserve">Check whether Kubernetes Service version is up-to-date</t>
   </si>
   <si>
-    <t xml:space="preserve">CM-7(a)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CM-8(1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CM-8(3)(a)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SA-3(a)</t>
+    <t xml:space="preserve">CM-07(a)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM-08(01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM-08(03)(a)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SA-03(a)</t>
   </si>
   <si>
     <t xml:space="preserve">IKS</t>
@@ -311,13 +311,13 @@
     <t xml:space="preserve">Check whether Continuous Delivery toolchain continuously scans source code to identify vulnerabilities above the # threshold. </t>
   </si>
   <si>
-    <t xml:space="preserve">RA-5(a) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SI-2(2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SI-7(1)</t>
+    <t xml:space="preserve">RA-05(a) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SI-02(02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SI-07(01)</t>
   </si>
   <si>
     <t xml:space="preserve">TOOLCHAIN</t>
@@ -470,84 +470,88 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -623,465 +627,571 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="0" width="39.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="20.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="24.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="1" width="39.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="20.98"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="R1" s="6"/>
-      <c r="S1" s="5" t="s">
+      <c r="R1" s="7"/>
+      <c r="S1" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
+      <c r="A2" s="8" t="n">
         <v>3000036</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="K2" s="11" t="s">
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="K2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="8" t="n">
         <v>3000109</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="13"/>
-      <c r="K3" s="11" t="s">
+      <c r="H3" s="14"/>
+      <c r="K3" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="L3" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10" t="s">
+      <c r="M3" s="11"/>
+      <c r="N3" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="O3" s="10"/>
-      <c r="P3" s="14" t="s">
+      <c r="O3" s="11"/>
+      <c r="P3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="Q3" s="10" t="s">
+      <c r="Q3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="R3" s="10"/>
-      <c r="S3" s="0" t="s">
+      <c r="R3" s="11"/>
+      <c r="S3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+    <row r="4" customFormat="false" ht="86.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="n">
         <v>3000110</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="13"/>
-      <c r="K4" s="11" t="s">
+      <c r="H4" s="14"/>
+      <c r="K4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="L4" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10" t="s">
+      <c r="M4" s="11"/>
+      <c r="N4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="10"/>
-      <c r="P4" s="14" t="s">
+      <c r="O4" s="11"/>
+      <c r="P4" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="Q4" s="10" t="s">
+      <c r="Q4" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="10"/>
-      <c r="S4" s="0" t="s">
+      <c r="R4" s="11"/>
+      <c r="S4" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="111.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+    <row r="5" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="n">
         <v>3000403</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="K5" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="L5" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10" t="s">
+      <c r="M5" s="11"/>
+      <c r="N5" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="O5" s="10"/>
-      <c r="P5" s="16" t="s">
+      <c r="O5" s="11"/>
+      <c r="P5" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="10"/>
-      <c r="S5" s="0" t="s">
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="8" t="n">
         <v>3000409</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10" t="s">
+      <c r="M6" s="11"/>
+      <c r="N6" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="O6" s="10"/>
-      <c r="P6" s="14" t="s">
+      <c r="O6" s="11"/>
+      <c r="P6" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="Q6" s="10" t="s">
+      <c r="Q6" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="R6" s="10"/>
+      <c r="R6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="8" t="n">
         <v>3000410</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10" t="s">
+      <c r="M7" s="11"/>
+      <c r="N7" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="0" t="s">
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11"/>
+      <c r="R7" s="11"/>
+      <c r="S7" s="1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="8" t="n">
         <v>3000450</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="K8" s="11" t="s">
+      <c r="K8" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10" t="s">
+      <c r="M8" s="11"/>
+      <c r="N8" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="144.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="8" t="n">
         <v>3000603</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="H9" s="10"/>
-      <c r="K9" s="18" t="s">
+      <c r="H9" s="11"/>
+      <c r="K9" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10" t="s">
+      <c r="M9" s="11"/>
+      <c r="N9" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="O9" s="10"/>
-      <c r="P9" s="16" t="s">
+      <c r="O9" s="11"/>
+      <c r="P9" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="Q9" s="19" t="s">
+      <c r="Q9" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="R9" s="19"/>
+      <c r="R9" s="20"/>
     </row>
-    <row r="10" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+    <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="n">
         <v>3000721</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="K10" s="11" t="s">
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="K10" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="L10" s="10" t="s">
+      <c r="L10" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10" t="s">
+      <c r="M10" s="11"/>
+      <c r="N10" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="73.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="8" t="n">
         <v>9000101</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="10"/>
-      <c r="K11" s="18" t="s">
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="11"/>
+      <c r="K11" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="L11" s="10" t="s">
+      <c r="L11" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10" t="s">
+      <c r="M11" s="11"/>
+      <c r="N11" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="O11" s="10"/>
-      <c r="P11" s="16" t="s">
+      <c r="O11" s="11"/>
+      <c r="P11" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="Q11" s="19" t="s">
+      <c r="Q11" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="R11" s="19"/>
+      <c r="R11" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1089,7 +1199,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>